<commit_message>
Update dashboard files and app
</commit_message>
<xml_diff>
--- a/MAS_Benchmarks.xlsx
+++ b/MAS_Benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ansalaza\mas-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{02D73E6E-9925-47AD-ACA6-00C4A3F49662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{94F6D4DC-B64C-4ECD-817A-E6EC2C15A2BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1390" yWindow="80" windowWidth="34320" windowHeight="13680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="140" windowWidth="32730" windowHeight="13040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark_Data" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="22">
   <si>
     <t>ManagerTeam</t>
   </si>
@@ -57,9 +57,6 @@
   </si>
   <si>
     <t>Seshu Chivukula</t>
-  </si>
-  <si>
-    <t>Willery Rivers</t>
   </si>
   <si>
     <t>Connie Serrano</t>
@@ -218,8 +215,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{71B9693B-4415-49D7-9582-118751D07E64}" name="tblBenchmarkData" displayName="tblBenchmarkData" ref="A1:E15" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="A1:E15" xr:uid="{71B9693B-4415-49D7-9582-118751D07E64}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{71B9693B-4415-49D7-9582-118751D07E64}" name="tblBenchmarkData" displayName="tblBenchmarkData" ref="A1:E14" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="A1:E14" xr:uid="{71B9693B-4415-49D7-9582-118751D07E64}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{184B8945-C042-4F94-9625-44B9911492BE}" name="ManagerTeam" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{F39D70CE-E74D-40F2-80E4-9FA1AF055671}" name="Associate Name" dataDxfId="3"/>
@@ -528,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
@@ -553,7 +550,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -561,7 +558,7 @@
         <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" s="1">
         <v>100</v>
@@ -570,7 +567,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -578,7 +575,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" s="1">
         <v>97.5</v>
@@ -587,7 +584,7 @@
         <v>2</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -595,7 +592,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1">
         <v>85.56</v>
@@ -604,7 +601,7 @@
         <v>3</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -612,7 +609,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" s="1">
         <v>80.709999999999994</v>
@@ -621,7 +618,7 @@
         <v>4</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -638,7 +635,7 @@
         <v>5</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -646,7 +643,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C7" s="1">
         <v>76.25</v>
@@ -655,7 +652,7 @@
         <v>6</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -663,7 +660,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C8" s="1">
         <v>71.25</v>
@@ -672,24 +669,24 @@
         <v>7</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="C9" s="1">
-        <v>59</v>
+        <v>100</v>
       </c>
       <c r="D9" s="1">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -697,16 +694,16 @@
         <v>5</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="C10" s="1">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="D10" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
@@ -714,16 +711,16 @@
         <v>5</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" s="1">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="D11" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -731,13 +728,13 @@
         <v>5</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C12" s="1">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D12" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>21</v>
@@ -748,16 +745,16 @@
         <v>5</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C13" s="1">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="D13" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -765,33 +762,16 @@
         <v>5</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C14" s="1">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D14" s="1">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="1">
-        <v>41</v>
-      </c>
-      <c r="D15" s="1">
-        <v>6</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -803,28 +783,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="081083fe-e475-436e-8ac6-57ab24d1081c" xsi:nil="true"/>
-    <Status xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Notes xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B7CF5D77C2318A48AE3D01AED053E969" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7f98047a509e9e082d0d58dfbe71352c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c3d3890c-cedb-4996-8d69-32a58562dce0" xmlns:ns3="081083fe-e475-436e-8ac6-57ab24d1081c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="361f48e45990901628f9319c45e78890" ns2:_="" ns3:_="">
     <xsd:import namespace="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
@@ -1075,32 +1033,29 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1678A2A8-E54E-4579-8501-27D3DA5E790E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98F52CCA-3969-42A2-9F3F-81FB4D653F1D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="081083fe-e475-436e-8ac6-57ab24d1081c" xsi:nil="true"/>
+    <Status xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Notes xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3AB7CB68-540E-4F04-820F-834558F23155}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1117,4 +1072,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98F52CCA-3969-42A2-9F3F-81FB4D653F1D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1678A2A8-E54E-4579-8501-27D3DA5E790E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Dashboard for Q1 Benchmarks and remove tracker/survey tabs
</commit_message>
<xml_diff>
--- a/MAS_Benchmarks.xlsx
+++ b/MAS_Benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ansalaza\mas-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94F6D4DC-B64C-4ECD-817A-E6EC2C15A2BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A861A9B-EBB7-4548-8C97-315C676A51EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="140" windowWidth="32730" windowHeight="13040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9600" yWindow="30" windowWidth="20210" windowHeight="13490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark_Data" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
   <si>
     <t>ManagerTeam</t>
   </si>
@@ -47,9 +47,6 @@
     <t>BenchmarkAverageScore</t>
   </si>
   <si>
-    <t>BenchmarkRank</t>
-  </si>
-  <si>
     <t>Charles</t>
   </si>
   <si>
@@ -95,13 +92,10 @@
     <t>Thomas Gordon</t>
   </si>
   <si>
-    <t>BenchmarkGroup</t>
-  </si>
-  <si>
-    <t>Top 20%</t>
-  </si>
-  <si>
-    <t>Bottom 20%</t>
+    <t>TyKee Walmsley</t>
+  </si>
+  <si>
+    <t>Willery Rivers</t>
   </si>
 </sst>
 </file>
@@ -145,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -153,17 +147,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="5">
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -215,14 +206,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{71B9693B-4415-49D7-9582-118751D07E64}" name="tblBenchmarkData" displayName="tblBenchmarkData" ref="A1:E14" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="A1:E14" xr:uid="{71B9693B-4415-49D7-9582-118751D07E64}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{184B8945-C042-4F94-9625-44B9911492BE}" name="ManagerTeam" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{F39D70CE-E74D-40F2-80E4-9FA1AF055671}" name="Associate Name" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{493C204F-90F3-43AF-93C9-1A6906233A17}" name="BenchmarkAverageScore" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{0AB553B9-16C6-453F-B1E2-1B4084C8EF4E}" name="BenchmarkRank" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{3C223DAB-4B57-4152-A6CF-3746484C3D9C}" name="BenchmarkGroup" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{71B9693B-4415-49D7-9582-118751D07E64}" name="tblBenchmarkData" displayName="tblBenchmarkData" ref="A1:C16" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="A1:C16" xr:uid="{71B9693B-4415-49D7-9582-118751D07E64}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{184B8945-C042-4F94-9625-44B9911492BE}" name="ManagerTeam" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{F39D70CE-E74D-40F2-80E4-9FA1AF055671}" name="Associate Name" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{493C204F-90F3-43AF-93C9-1A6906233A17}" name="BenchmarkAverageScore" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -525,18 +514,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.54296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.7265625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="26.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -546,232 +533,170 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C2" s="1">
         <v>100</v>
       </c>
-      <c r="D2" s="1">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C3" s="1">
-        <v>97.5</v>
-      </c>
-      <c r="D3" s="1">
-        <v>2</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+        <v>97.78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1">
         <v>85.56</v>
       </c>
-      <c r="D4" s="1">
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="1">
+        <v>73.89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="1">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1">
+        <v>67.78</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="1">
+        <v>74.44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1">
-        <v>80.709999999999994</v>
-      </c>
-      <c r="D5" s="1">
-        <v>4</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="1">
-        <v>77.78</v>
-      </c>
-      <c r="D6" s="1">
-        <v>5</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" s="1">
-        <v>76.25</v>
-      </c>
-      <c r="D7" s="1">
-        <v>6</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="1">
-        <v>71.25</v>
-      </c>
-      <c r="D8" s="1">
-        <v>7</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>5</v>
-      </c>
       <c r="B9" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" s="1">
         <v>100</v>
       </c>
-      <c r="D9" s="1">
-        <v>1</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C10" s="1">
         <v>79</v>
       </c>
-      <c r="D10" s="1">
-        <v>2</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C11" s="1">
         <v>65</v>
       </c>
-      <c r="D11" s="1">
-        <v>3</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" s="1">
         <v>55</v>
       </c>
-      <c r="D12" s="1">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>5</v>
-      </c>
       <c r="B13" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" s="1">
         <v>44</v>
       </c>
-      <c r="D13" s="1">
-        <v>5</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C14" s="1">
         <v>41</v>
       </c>
-      <c r="D14" s="1">
-        <v>6</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>21</v>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="1">
+        <v>96.67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="1">
+        <v>53.64</v>
       </c>
     </row>
   </sheetData>
@@ -783,6 +708,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B7CF5D77C2318A48AE3D01AED053E969" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7f98047a509e9e082d0d58dfbe71352c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c3d3890c-cedb-4996-8d69-32a58562dce0" xmlns:ns3="081083fe-e475-436e-8ac6-57ab24d1081c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="361f48e45990901628f9319c45e78890" ns2:_="" ns3:_="">
     <xsd:import namespace="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
@@ -1033,15 +967,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1056,6 +981,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98F52CCA-3969-42A2-9F3F-81FB4D653F1D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3AB7CB68-540E-4F04-820F-834558F23155}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1074,14 +1007,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98F52CCA-3969-42A2-9F3F-81FB4D653F1D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1678A2A8-E54E-4579-8501-27D3DA5E790E}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update MAS call grading raw data
</commit_message>
<xml_diff>
--- a/MAS_Benchmarks.xlsx
+++ b/MAS_Benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ansalaza\mas-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD131D0D-AF21-49A3-BDDB-31A70E0D1FA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{413A117F-B0BD-45C0-962E-F6D60D29CC04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1800" yWindow="190" windowWidth="29960" windowHeight="13490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1780" yWindow="370" windowWidth="29960" windowHeight="13490" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Benchmark_Data" sheetId="1" r:id="rId1"/>
@@ -705,16 +705,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="081083fe-e475-436e-8ac6-57ab24d1081c" xsi:nil="true"/>
-    <Status xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Notes xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -969,27 +965,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="081083fe-e475-436e-8ac6-57ab24d1081c" xsi:nil="true"/>
+    <Status xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Notes xmlns="c3d3890c-cedb-4996-8d69-32a58562dce0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1678A2A8-E54E-4579-8501-27D3DA5E790E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98F52CCA-3969-42A2-9F3F-81FB4D653F1D}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1014,9 +1005,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98F52CCA-3969-42A2-9F3F-81FB4D653F1D}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1678A2A8-E54E-4579-8501-27D3DA5E790E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="081083fe-e475-436e-8ac6-57ab24d1081c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="c3d3890c-cedb-4996-8d69-32a58562dce0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>